<commit_message>
corrected specs and components uploaded
</commit_message>
<xml_diff>
--- a/MATERIALS/Specs and components.xlsx
+++ b/MATERIALS/Specs and components.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/21a80410d6fdd5b9/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="114" documentId="8_{6EC2E1DA-13C4-4F83-AF77-9D5EB2763161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15887EFA-BCB1-462E-913B-FD16C28C4139}"/>
+  <xr:revisionPtr revIDLastSave="116" documentId="8_{6EC2E1DA-13C4-4F83-AF77-9D5EB2763161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{79D9EE55-6BF9-4DF8-8359-1079CA140B56}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{933BEE87-A7D3-4027-87E5-EDDCFEEC1D3D}"/>
   </bookViews>
@@ -165,9 +165,6 @@
     <t>AP2112K-3.3</t>
   </si>
   <si>
-    <t>Passives, headers, switch, button</t>
-  </si>
-  <si>
     <t>Mixed</t>
   </si>
   <si>
@@ -203,12 +200,6 @@
 Fixed address 0x57</t>
   </si>
   <si>
-    <t>Onboard voltage regulator 
-Onboard pull-up resistors on SDA/SCL
-AD0 pin tied to a defined level (not left floating) 
-Default address 0x68 (confirm AD0 wiring gives you this)</t>
-  </si>
-  <si>
     <t>Confirm it’s the classic ESP32-WROOM-32 based DevKit V1 (not an S2/S3/C3 variant)
 Has a USB port for programming (most do, but double-check it’s not a bare module requiring separate programming hardware)</t>
   </si>
@@ -228,6 +219,15 @@
   </si>
   <si>
     <t>Confirm it’s specifically the 3.3V output version (AP2112K is sold in multiple fixed-voltage versions: 3.3V, 2.5V, 1.8V, etc. so the exact part number suffix matters; something like “AP2112K-3.3” )</t>
+  </si>
+  <si>
+    <t>Passives, headers, switch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onboard voltage regulator 
+Onboard pull-up resistors on SDA/SCL
+AD0 pin tied to a defined level (not left floating) 
+Default address 0x68 </t>
   </si>
 </sst>
 </file>
@@ -300,12 +300,6 @@
   </cellStyles>
   <dxfs count="11">
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -335,6 +329,12 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -377,17 +377,13 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1481C852-91E6-4AD8-B11E-AB54B2892A94}" name="Table1" displayName="Table1" ref="A1:C9" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1481C852-91E6-4AD8-B11E-AB54B2892A94}" name="Table1" displayName="Table1" ref="A1:C9" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
   <autoFilter ref="A1:C9" xr:uid="{1481C852-91E6-4AD8-B11E-AB54B2892A94}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{553235B5-9EFF-49A8-864D-045425C7DB39}" name="Parameter" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{AF491593-D60C-406C-A3AD-19AFFCBE6313}" name="Target" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{4874F35F-0EEE-4EB7-94A4-05D9B05F5EC6}" name="Hardware" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{553235B5-9EFF-49A8-864D-045425C7DB39}" name="Parameter" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{AF491593-D60C-406C-A3AD-19AFFCBE6313}" name="Target" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{4874F35F-0EEE-4EB7-94A4-05D9B05F5EC6}" name="Hardware" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -399,8 +395,8 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{520E3EAA-09EA-48E0-A539-1B3914A29811}" name="Component" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{8ADCAF73-F750-4C94-B106-70CF37E9C818}" name="Part" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{F6E79DF3-FE4E-46A6-90BE-87710729560C}" name="Qty" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{2BBEBA9A-C2DC-45C3-8FA7-1D6E5F9A55DF}" name="Must contain" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{F6E79DF3-FE4E-46A6-90BE-87710729560C}" name="Qty" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{2BBEBA9A-C2DC-45C3-8FA7-1D6E5F9A55DF}" name="Must contain" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -851,7 +847,7 @@
         <v>26</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="3" customFormat="1" ht="81" customHeight="1" x14ac:dyDescent="0.3">
@@ -865,7 +861,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="3" customFormat="1" ht="67.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -879,7 +875,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="3" customFormat="1" ht="103.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -893,7 +889,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="3" customFormat="1" ht="97.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -907,7 +903,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="3" customFormat="1" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -921,7 +917,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:4" s="3" customFormat="1" ht="131.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -935,7 +931,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:4" s="3" customFormat="1" ht="65.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
@@ -949,7 +945,7 @@
         <v>1</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:4" s="3" customFormat="1" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -963,27 +959,27 @@
         <v>1</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="3" customFormat="1" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>44</v>
       </c>
       <c r="D10" s="5"/>
     </row>
     <row r="11" spans="1:4" s="3" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>46</v>
       </c>
       <c r="C11" s="1">
         <v>5</v>
@@ -992,10 +988,10 @@
     </row>
     <row r="12" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>48</v>
       </c>
       <c r="C12" s="1">
         <v>1</v>

</xml_diff>